<commit_message>
add one guide Laura
</commit_message>
<xml_diff>
--- a/Control Guias Silvia.xlsx
+++ b/Control Guias Silvia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAMBRIZ\Desktop\Proyectos\Capacitaciones\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51815C41-70FD-4CAD-8B00-E1286EBCA047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09FA75E-8123-4D65-B306-071B5257A61B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{28D40DE8-55EE-4A45-8730-C507FE790F49}"/>
+    <workbookView xWindow="1440" yWindow="-16335" windowWidth="29070" windowHeight="15750" xr2:uid="{28D40DE8-55EE-4A45-8730-C507FE790F49}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="48">
   <si>
     <t>YADIRA ANDRADE HERRERA</t>
   </si>
@@ -168,6 +168,15 @@
   </si>
   <si>
     <t>1055898160612700749507</t>
+  </si>
+  <si>
+    <t>Laura Sedano Gonzalez</t>
+  </si>
+  <si>
+    <t>2026-09-30 12:23:15.0</t>
+  </si>
+  <si>
+    <t>3055898160612700749520</t>
   </si>
 </sst>
 </file>
@@ -801,81 +810,10 @@
   </cellStyles>
   <dxfs count="23">
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="7"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Poppinsregular"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color rgb="FFD1D1D1"/>
-        </left>
-        <right style="medium">
-          <color rgb="FFD1D1D1"/>
-        </right>
-        <top style="medium">
-          <color rgb="FFD1D1D1"/>
-        </top>
-        <bottom style="medium">
-          <color rgb="FFD1D1D1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="7"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Poppinsregular"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FFD1D1D1"/>
-        </left>
-        <right style="medium">
-          <color rgb="FFD1D1D1"/>
-        </right>
-        <top style="medium">
-          <color rgb="FFD1D1D1"/>
-        </top>
-        <bottom/>
-      </border>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
       <font>
@@ -952,10 +890,41 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Poppinsregular"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFD1D1D1"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFD1D1D1"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFD1D1D1"/>
+        </top>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1277,6 +1246,46 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Poppinsregular"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color rgb="FFD1D1D1"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFD1D1D1"/>
+        </right>
+        <top style="medium">
+          <color rgb="FFD1D1D1"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FFD1D1D1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
         <sz val="8.25"/>
         <color rgb="FF525252"/>
         <name val="Poppinsregular"/>
@@ -1524,8 +1533,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{490D4088-391A-4561-A356-EB3A167A3CB4}" name="Tabla1" displayName="Tabla1" ref="A1:K26" totalsRowCount="1" headerRowDxfId="22">
-  <autoFilter ref="A1:K25" xr:uid="{490D4088-391A-4561-A356-EB3A167A3CB4}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{490D4088-391A-4561-A356-EB3A167A3CB4}" name="Tabla1" displayName="Tabla1" ref="A1:K27" totalsRowCount="1" headerRowDxfId="22">
+  <autoFilter ref="A1:K26" xr:uid="{490D4088-391A-4561-A356-EB3A167A3CB4}">
     <filterColumn colId="2">
       <filters>
         <filter val="Alberto Alonso Figueroa"/>
@@ -1547,22 +1556,22 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4B063840-E3E0-424F-895C-FE9BEF01A625}" name="ID" dataDxfId="21" totalsRowDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{AF0F79CD-D3FD-459E-975B-73126EC45FBF}" name="REMITENTE" dataDxfId="20" totalsRowDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{C3021A36-4783-4A00-B0D1-6D03B6593DFB}" name="DESTINATARIO" dataDxfId="19" totalsRowDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{D9C6EAF9-70E7-4707-806A-CE080DF20389}" name="PAQUETERIA" dataDxfId="18" totalsRowDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{6610E46E-6520-4A33-B1D8-FEA7DAEC3BC5}" name="FECHA" dataDxfId="17" totalsRowDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{E3F30373-116B-4AED-9C5A-E915D0CA490A}" name="GUIA\" dataDxfId="16" totalsRowDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{A8BCC94E-A2E1-4681-BCB0-2660B2337655}" name="Columna1" dataDxfId="0" totalsRowDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{CF67D91C-74D6-40D6-BF1E-CA5ED94ED0EE}" name="COSTO" dataDxfId="15" totalsRowDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{CD5147F2-4A45-429E-B161-2095B3278722}" name="PRECIO" totalsRowFunction="custom" dataDxfId="14" totalsRowDxfId="2">
+    <tableColumn id="1" xr3:uid="{4B063840-E3E0-424F-895C-FE9BEF01A625}" name="ID" dataDxfId="21" totalsRowDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{AF0F79CD-D3FD-459E-975B-73126EC45FBF}" name="REMITENTE" dataDxfId="20" totalsRowDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{C3021A36-4783-4A00-B0D1-6D03B6593DFB}" name="DESTINATARIO" dataDxfId="19" totalsRowDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{D9C6EAF9-70E7-4707-806A-CE080DF20389}" name="PAQUETERIA" dataDxfId="18" totalsRowDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{6610E46E-6520-4A33-B1D8-FEA7DAEC3BC5}" name="FECHA" dataDxfId="17" totalsRowDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{E3F30373-116B-4AED-9C5A-E915D0CA490A}" name="GUIA\" dataDxfId="16" totalsRowDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{A8BCC94E-A2E1-4681-BCB0-2660B2337655}" name="Columna1" dataDxfId="15" totalsRowDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{CF67D91C-74D6-40D6-BF1E-CA5ED94ED0EE}" name="COSTO" dataDxfId="14" totalsRowDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{CD5147F2-4A45-429E-B161-2095B3278722}" name="PRECIO" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="2">
       <calculatedColumnFormula>Tabla1[[#This Row],[COSTO]]+50</calculatedColumnFormula>
-      <totalsRowFormula>SUBTOTAL(9,I2:I25)</totalsRowFormula>
+      <totalsRowFormula>SUBTOTAL(9,I2:I26)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A225C977-ACF0-40F2-8505-790183442B8A}" name="SALDO" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="5">
-      <totalsRowFormula>SUBTOTAL(9,J2:J25)</totalsRowFormula>
+    <tableColumn id="10" xr3:uid="{A225C977-ACF0-40F2-8505-790183442B8A}" name="SALDO" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="1">
+      <totalsRowFormula>SUBTOTAL(9,J2:J26)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{FD3FBAD4-BE3D-4E04-82AF-D6DAF9FBBD62}" name="RESTO" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="4">
+    <tableColumn id="11" xr3:uid="{FD3FBAD4-BE3D-4E04-82AF-D6DAF9FBBD62}" name="RESTO" totalsRowFunction="custom" dataDxfId="11" totalsRowDxfId="0">
       <totalsRowFormula>Tabla1[[#Totals],[SALDO]]-Tabla1[[#Totals],[PRECIO]]</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -1887,7 +1896,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A89A7B97-BC33-4D79-8675-A33F022C66EB}">
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="5" hidden="1" customWidth="1"/>
@@ -1942,23 +1951,23 @@
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H2" s="13">
-        <v>271</v>
+        <v>376</v>
       </c>
       <c r="I2" s="11">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>321</v>
+        <v>426</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1972,10 +1981,10 @@
         <v>2</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H3" s="13">
         <v>271</v>
@@ -1990,18 +1999,18 @@
         <v>0</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H4" s="15">
+        <v>44</v>
+      </c>
+      <c r="H4" s="13">
         <v>271</v>
       </c>
       <c r="I4" s="11">
@@ -2009,7 +2018,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15" thickBot="1">
+    <row r="5" spans="1:11">
       <c r="B5" s="5" t="s">
         <v>0</v>
       </c>
@@ -2020,105 +2029,95 @@
         <v>2</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H5" s="15">
-        <v>231</v>
+        <v>271</v>
       </c>
       <c r="I5" s="11">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>281</v>
+        <v>321</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15" thickBot="1">
-      <c r="A6" s="1">
-        <v>2318020</v>
-      </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="C6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="2">
-        <v>46289.487349537034</v>
-      </c>
-      <c r="F6" s="1">
-        <v>5.0558981606126995E+21</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="H6" s="14">
-        <v>167</v>
-      </c>
-      <c r="I6" s="9">
+      <c r="E6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" s="15">
+        <v>231</v>
+      </c>
+      <c r="I6" s="11">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>217</v>
-      </c>
-      <c r="J6" s="11">
-        <v>318</v>
-      </c>
-      <c r="K6" s="11"/>
+        <v>281</v>
+      </c>
     </row>
     <row r="7" spans="1:11" ht="15" thickBot="1">
       <c r="A7" s="1">
-        <v>2317843</v>
+        <v>2318020</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E7" s="2">
-        <v>46289.440324074072</v>
+        <v>46289.487349537034</v>
       </c>
       <c r="F7" s="1">
-        <v>4.0559097447817198E+21</v>
+        <v>5.0558981606126995E+21</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>3</v>
       </c>
       <c r="H7" s="14">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="I7" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="J7" s="11">
-        <v>5000</v>
+        <v>318</v>
       </c>
       <c r="K7" s="11"/>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
       <c r="A8" s="1">
-        <v>2316890</v>
+        <v>2317843</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E8" s="2">
-        <v>46288.584930555553</v>
+        <v>46289.440324074072</v>
       </c>
       <c r="F8" s="1">
-        <v>3.0559097447817198E+21</v>
+        <v>4.0559097447817198E+21</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>3</v>
@@ -2130,27 +2129,29 @@
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
         <v>205</v>
       </c>
-      <c r="J8" s="11"/>
+      <c r="J8" s="11">
+        <v>5000</v>
+      </c>
       <c r="K8" s="11"/>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1">
       <c r="A9" s="1">
-        <v>2316880</v>
+        <v>2316890</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E9" s="2">
-        <v>46288.58326388889</v>
+        <v>46288.584930555553</v>
       </c>
       <c r="F9" s="1">
-        <v>9.0559097447817203E+21</v>
+        <v>3.0559097447817198E+21</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>3</v>
@@ -2165,327 +2166,327 @@
       <c r="J9" s="11"/>
       <c r="K9" s="11"/>
     </row>
-    <row r="10" spans="1:11" ht="22.2" hidden="1" thickBot="1">
+    <row r="10" spans="1:11" ht="15" thickBot="1">
       <c r="A10" s="1">
-        <v>2314309</v>
+        <v>2316880</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10" s="2">
+        <v>46288.58326388889</v>
+      </c>
+      <c r="F10" s="1">
+        <v>9.0559097447817203E+21</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H10" s="14">
+        <v>155</v>
+      </c>
+      <c r="I10" s="9">
+        <f>Tabla1[[#This Row],[COSTO]]+50</f>
+        <v>205</v>
+      </c>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+    </row>
+    <row r="11" spans="1:11" ht="22.2" hidden="1" thickBot="1">
+      <c r="A11" s="1">
+        <v>2314309</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E11" s="2">
         <v>46287.342395833337</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F11" s="1">
         <v>2.0558981606127001E+21</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H11" s="1">
         <v>271</v>
       </c>
-      <c r="I10" s="4">
+      <c r="I11" s="4">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
         <v>321</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="39" thickBot="1">
-      <c r="A11" s="1">
+    <row r="12" spans="1:11" ht="39" thickBot="1">
+      <c r="A12" s="1">
         <v>2313907</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E12" s="2">
         <v>46286.680763888886</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F12" s="1">
         <v>3.0558981606127001E+21</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H11" s="14">
+      <c r="H12" s="14">
         <v>164</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I12" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
         <v>214</v>
-      </c>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-    </row>
-    <row r="12" spans="1:11" ht="58.2" thickBot="1">
-      <c r="A12" s="1">
-        <v>2312903</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" s="2">
-        <v>46286.505462962959</v>
-      </c>
-      <c r="F12" s="1">
-        <v>5.5898160612700701E+19</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="14">
-        <v>310</v>
-      </c>
-      <c r="I12" s="9">
-        <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>360</v>
       </c>
       <c r="J12" s="11"/>
       <c r="K12" s="11"/>
     </row>
     <row r="13" spans="1:11" ht="58.2" thickBot="1">
       <c r="A13" s="1">
-        <v>2312796</v>
+        <v>2312903</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E13" s="2">
-        <v>46286.48704861111</v>
+        <v>46286.505462962959</v>
       </c>
       <c r="F13" s="1">
-        <v>3.0559097447817198E+21</v>
+        <v>5.5898160612700701E+19</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H13" s="14">
-        <v>155</v>
+        <v>310</v>
       </c>
       <c r="I13" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>205</v>
+        <v>360</v>
       </c>
       <c r="J13" s="11"/>
       <c r="K13" s="11"/>
     </row>
-    <row r="14" spans="1:11" ht="15" thickBot="1">
+    <row r="14" spans="1:11" ht="58.2" thickBot="1">
       <c r="A14" s="1">
-        <v>2309136</v>
+        <v>2312796</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E14" s="2">
-        <v>46282.538715277777</v>
+        <v>46286.48704861111</v>
       </c>
       <c r="F14" s="1">
-        <v>5.0558981606126995E+21</v>
+        <v>3.0559097447817198E+21</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H14" s="14">
-        <v>190</v>
+        <v>155</v>
       </c>
       <c r="I14" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="J14" s="11"/>
       <c r="K14" s="11"/>
     </row>
     <row r="15" spans="1:11" ht="15" thickBot="1">
       <c r="A15" s="1">
-        <v>2308942</v>
+        <v>2309136</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E15" s="2">
-        <v>46282.501782407409</v>
+        <v>46282.538715277777</v>
       </c>
       <c r="F15" s="1">
-        <v>6.0558981606126995E+21</v>
+        <v>5.0558981606126995E+21</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H15" s="14">
-        <v>229</v>
+        <v>190</v>
       </c>
       <c r="I15" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="J15" s="11"/>
       <c r="K15" s="11"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
       <c r="A16" s="1">
-        <v>2308752</v>
+        <v>2308942</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E16" s="2">
-        <v>46282.467881944445</v>
+        <v>46282.501782407409</v>
       </c>
       <c r="F16" s="1">
-        <v>9.0558981606126995E+21</v>
+        <v>6.0558981606126995E+21</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H16" s="14">
-        <v>179</v>
+        <v>229</v>
       </c>
       <c r="I16" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>229</v>
+        <v>279</v>
       </c>
       <c r="J16" s="11"/>
       <c r="K16" s="11"/>
     </row>
     <row r="17" spans="1:11" ht="15" thickBot="1">
       <c r="A17" s="1">
-        <v>2308664</v>
+        <v>2308752</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E17" s="2">
-        <v>46282.450474537036</v>
+        <v>46282.467881944445</v>
       </c>
       <c r="F17" s="1">
-        <v>1.0558981606127001E+21</v>
+        <v>9.0558981606126995E+21</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H17" s="14">
-        <v>229</v>
+        <v>179</v>
       </c>
       <c r="I17" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>279</v>
+        <v>229</v>
       </c>
       <c r="J17" s="11"/>
       <c r="K17" s="11"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
       <c r="A18" s="1">
-        <v>2307450</v>
+        <v>2308664</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E18" s="2">
-        <v>46280.594768518517</v>
+        <v>46282.450474537036</v>
       </c>
       <c r="F18" s="1">
-        <v>8.0558981606126995E+21</v>
+        <v>1.0558981606127001E+21</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H18" s="14">
-        <v>271</v>
+        <v>229</v>
       </c>
       <c r="I18" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>321</v>
+        <v>279</v>
       </c>
       <c r="J18" s="11"/>
       <c r="K18" s="11"/>
     </row>
     <row r="19" spans="1:11" ht="15" thickBot="1">
       <c r="A19" s="1">
-        <v>2307446</v>
+        <v>2307450</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E19" s="2">
-        <v>46280.593831018516</v>
+        <v>46280.594768518517</v>
       </c>
       <c r="F19" s="1">
-        <v>5.5898160612700701E+19</v>
+        <v>8.0558981606126995E+21</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H19" s="14">
-        <v>302</v>
+        <v>271</v>
       </c>
       <c r="I19" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>352</v>
+        <v>321</v>
       </c>
       <c r="J19" s="11"/>
       <c r="K19" s="11"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
       <c r="A20" s="1">
-        <v>2307438</v>
+        <v>2307446</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>0</v>
@@ -2497,10 +2498,10 @@
         <v>2</v>
       </c>
       <c r="E20" s="2">
-        <v>46280.591377314813</v>
+        <v>46280.593831018516</v>
       </c>
       <c r="F20" s="1">
-        <v>4.0558981606127001E+21</v>
+        <v>5.5898160612700701E+19</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>9</v>
@@ -2517,133 +2518,133 @@
     </row>
     <row r="21" spans="1:11" ht="15" thickBot="1">
       <c r="A21" s="1">
-        <v>2304456</v>
+        <v>2307438</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E21" s="2">
-        <v>46279.455949074072</v>
+        <v>46280.591377314813</v>
       </c>
       <c r="F21" s="1">
-        <v>3.0558981606127001E+21</v>
+        <v>4.0558981606127001E+21</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H21" s="14">
-        <v>179</v>
+        <v>302</v>
       </c>
       <c r="I21" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>229</v>
+        <v>352</v>
       </c>
       <c r="J21" s="11"/>
       <c r="K21" s="11"/>
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
       <c r="A22" s="1">
-        <v>2304430</v>
+        <v>2304456</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E22" s="2">
-        <v>46279.4528125</v>
+        <v>46279.455949074072</v>
       </c>
       <c r="F22" s="1">
-        <v>9.0558981606126995E+21</v>
+        <v>3.0558981606127001E+21</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H22" s="14">
-        <v>414</v>
+        <v>179</v>
       </c>
       <c r="I22" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>464</v>
+        <v>229</v>
       </c>
       <c r="J22" s="11"/>
       <c r="K22" s="11"/>
     </row>
-    <row r="23" spans="1:11" ht="22.2" hidden="1" thickBot="1">
+    <row r="23" spans="1:11" ht="15" thickBot="1">
       <c r="A23" s="1">
-        <v>2303299</v>
+        <v>2304430</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E23" s="2">
+        <v>46279.4528125</v>
+      </c>
+      <c r="F23" s="1">
+        <v>9.0558981606126995E+21</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H23" s="14">
+        <v>414</v>
+      </c>
+      <c r="I23" s="9">
+        <f>Tabla1[[#This Row],[COSTO]]+50</f>
+        <v>464</v>
+      </c>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+    </row>
+    <row r="24" spans="1:11" ht="22.2" hidden="1" thickBot="1">
+      <c r="A24" s="1">
+        <v>2303299</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E24" s="2">
         <v>46277.375405092593</v>
       </c>
-      <c r="F23" s="1">
+      <c r="F24" s="1">
         <v>8.0558981606126995E+21</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G24" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H24" s="1">
         <v>271</v>
       </c>
-      <c r="I23" s="4">
+      <c r="I24" s="4">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
         <v>321</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" ht="15" thickBot="1">
-      <c r="A24" s="1">
-        <v>2302573</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E24" s="2">
-        <v>46276.538518518515</v>
-      </c>
-      <c r="F24" s="1">
-        <v>3.0558981606127001E+21</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H24" s="14">
-        <v>302</v>
-      </c>
-      <c r="I24" s="9">
-        <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>352</v>
-      </c>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
     </row>
     <row r="25" spans="1:11" ht="15" thickBot="1">
       <c r="A25" s="1">
-        <v>2302572</v>
+        <v>2302573</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>0</v>
@@ -2655,10 +2656,10 @@
         <v>2</v>
       </c>
       <c r="E25" s="2">
-        <v>46276.53769675926</v>
+        <v>46276.538518518515</v>
       </c>
       <c r="F25" s="1">
-        <v>5.0558981606126995E+21</v>
+        <v>3.0558981606127001E+21</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>9</v>
@@ -2666,33 +2667,65 @@
       <c r="H25" s="14">
         <v>302</v>
       </c>
-      <c r="I25" s="10">
+      <c r="I25" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
         <v>352</v>
       </c>
       <c r="J25" s="11"/>
       <c r="K25" s="11"/>
     </row>
-    <row r="26" spans="1:11">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="17">
-        <f>SUBTOTAL(9,I2:I25)</f>
-        <v>6304</v>
-      </c>
-      <c r="J26" s="12">
-        <f>SUBTOTAL(9,J2:J25)</f>
+    <row r="26" spans="1:11" ht="15" thickBot="1">
+      <c r="A26" s="1">
+        <v>2302572</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26" s="2">
+        <v>46276.53769675926</v>
+      </c>
+      <c r="F26" s="1">
+        <v>5.0558981606126995E+21</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H26" s="14">
+        <v>302</v>
+      </c>
+      <c r="I26" s="10">
+        <f>Tabla1[[#This Row],[COSTO]]+50</f>
+        <v>352</v>
+      </c>
+      <c r="J26" s="11"/>
+      <c r="K26" s="11"/>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="17">
+        <f>SUBTOTAL(9,I2:I26)</f>
+        <v>6730</v>
+      </c>
+      <c r="J27" s="12">
+        <f>SUBTOTAL(9,J2:J26)</f>
         <v>5318</v>
       </c>
-      <c r="K26" s="12">
+      <c r="K27" s="12">
         <f>Tabla1[[#Totals],[SALDO]]-Tabla1[[#Totals],[PRECIO]]</f>
-        <v>-986</v>
+        <v>-1412</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add Osvaldo Sayavedra guide
</commit_message>
<xml_diff>
--- a/Control Guias Silvia.xlsx
+++ b/Control Guias Silvia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAMBRIZ\Desktop\Proyectos\Capacitaciones\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09FA75E-8123-4D65-B306-071B5257A61B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65F4BE49-99E3-4D62-9F4B-3E2FB4818D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1440" yWindow="-16335" windowWidth="29070" windowHeight="15750" xr2:uid="{28D40DE8-55EE-4A45-8730-C507FE790F49}"/>
+    <workbookView xWindow="1455" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{28D40DE8-55EE-4A45-8730-C507FE790F49}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="51">
   <si>
     <t>YADIRA ANDRADE HERRERA</t>
   </si>
@@ -177,6 +177,15 @@
   </si>
   <si>
     <t>3055898160612700749520</t>
+  </si>
+  <si>
+    <t>Osvaldo Sayavedra Carmona</t>
+  </si>
+  <si>
+    <t>4055898160612700749652</t>
+  </si>
+  <si>
+    <t>2026-10-02 11:16:22.0</t>
   </si>
 </sst>
 </file>
@@ -1533,8 +1542,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{490D4088-391A-4561-A356-EB3A167A3CB4}" name="Tabla1" displayName="Tabla1" ref="A1:K27" totalsRowCount="1" headerRowDxfId="22">
-  <autoFilter ref="A1:K26" xr:uid="{490D4088-391A-4561-A356-EB3A167A3CB4}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{490D4088-391A-4561-A356-EB3A167A3CB4}" name="Tabla1" displayName="Tabla1" ref="A1:K28" totalsRowCount="1" headerRowDxfId="22">
+  <autoFilter ref="A1:K27" xr:uid="{490D4088-391A-4561-A356-EB3A167A3CB4}">
     <filterColumn colId="2">
       <filters>
         <filter val="Alberto Alonso Figueroa"/>
@@ -1566,10 +1575,10 @@
     <tableColumn id="8" xr3:uid="{CF67D91C-74D6-40D6-BF1E-CA5ED94ED0EE}" name="COSTO" dataDxfId="14" totalsRowDxfId="3"/>
     <tableColumn id="9" xr3:uid="{CD5147F2-4A45-429E-B161-2095B3278722}" name="PRECIO" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="2">
       <calculatedColumnFormula>Tabla1[[#This Row],[COSTO]]+50</calculatedColumnFormula>
-      <totalsRowFormula>SUBTOTAL(9,I2:I26)</totalsRowFormula>
+      <totalsRowFormula>SUBTOTAL(9,I2:I27)</totalsRowFormula>
     </tableColumn>
     <tableColumn id="10" xr3:uid="{A225C977-ACF0-40F2-8505-790183442B8A}" name="SALDO" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="1">
-      <totalsRowFormula>SUBTOTAL(9,J2:J26)</totalsRowFormula>
+      <totalsRowFormula>SUBTOTAL(9,J2:J27)</totalsRowFormula>
     </tableColumn>
     <tableColumn id="11" xr3:uid="{FD3FBAD4-BE3D-4E04-82AF-D6DAF9FBBD62}" name="RESTO" totalsRowFunction="custom" dataDxfId="11" totalsRowDxfId="0">
       <totalsRowFormula>Tabla1[[#Totals],[SALDO]]-Tabla1[[#Totals],[PRECIO]]</totalsRowFormula>
@@ -1896,7 +1905,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A89A7B97-BC33-4D79-8675-A33F022C66EB}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="5" hidden="1" customWidth="1"/>
@@ -1951,23 +1960,23 @@
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H2" s="13">
-        <v>376</v>
+        <v>177</v>
       </c>
       <c r="I2" s="11">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>426</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1975,23 +1984,23 @@
         <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H3" s="13">
-        <v>271</v>
+        <v>376</v>
       </c>
       <c r="I3" s="11">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>321</v>
+        <v>426</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -2005,10 +2014,10 @@
         <v>2</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H4" s="13">
         <v>271</v>
@@ -2023,18 +2032,18 @@
         <v>0</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="15">
+        <v>44</v>
+      </c>
+      <c r="H5" s="13">
         <v>271</v>
       </c>
       <c r="I5" s="11">
@@ -2042,7 +2051,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15" thickBot="1">
+    <row r="6" spans="1:11">
       <c r="B6" s="5" t="s">
         <v>0</v>
       </c>
@@ -2053,105 +2062,95 @@
         <v>2</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H6" s="15">
-        <v>231</v>
+        <v>271</v>
       </c>
       <c r="I6" s="11">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>281</v>
+        <v>321</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15" thickBot="1">
-      <c r="A7" s="1">
-        <v>2318020</v>
-      </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D7" s="1" t="s">
+      <c r="C7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="2">
-        <v>46289.487349537034</v>
-      </c>
-      <c r="F7" s="1">
-        <v>5.0558981606126995E+21</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="H7" s="14">
-        <v>167</v>
-      </c>
-      <c r="I7" s="9">
+      <c r="E7" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" s="15">
+        <v>231</v>
+      </c>
+      <c r="I7" s="11">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>217</v>
-      </c>
-      <c r="J7" s="11">
-        <v>318</v>
-      </c>
-      <c r="K7" s="11"/>
+        <v>281</v>
+      </c>
     </row>
     <row r="8" spans="1:11" ht="15" thickBot="1">
       <c r="A8" s="1">
-        <v>2317843</v>
+        <v>2318020</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E8" s="2">
-        <v>46289.440324074072</v>
+        <v>46289.487349537034</v>
       </c>
       <c r="F8" s="1">
-        <v>4.0559097447817198E+21</v>
+        <v>5.0558981606126995E+21</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="H8" s="14">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="I8" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="J8" s="11">
-        <v>5000</v>
+        <v>318</v>
       </c>
       <c r="K8" s="11"/>
     </row>
     <row r="9" spans="1:11" ht="15" thickBot="1">
       <c r="A9" s="1">
-        <v>2316890</v>
+        <v>2317843</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E9" s="2">
-        <v>46288.584930555553</v>
+        <v>46289.440324074072</v>
       </c>
       <c r="F9" s="1">
-        <v>3.0559097447817198E+21</v>
+        <v>4.0559097447817198E+21</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>3</v>
@@ -2163,27 +2162,29 @@
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
         <v>205</v>
       </c>
-      <c r="J9" s="11"/>
+      <c r="J9" s="11">
+        <v>5000</v>
+      </c>
       <c r="K9" s="11"/>
     </row>
     <row r="10" spans="1:11" ht="15" thickBot="1">
       <c r="A10" s="1">
-        <v>2316880</v>
+        <v>2316890</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E10" s="2">
-        <v>46288.58326388889</v>
+        <v>46288.584930555553</v>
       </c>
       <c r="F10" s="1">
-        <v>9.0559097447817203E+21</v>
+        <v>3.0559097447817198E+21</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>3</v>
@@ -2198,327 +2199,327 @@
       <c r="J10" s="11"/>
       <c r="K10" s="11"/>
     </row>
-    <row r="11" spans="1:11" ht="22.2" hidden="1" thickBot="1">
+    <row r="11" spans="1:11" ht="15" thickBot="1">
       <c r="A11" s="1">
-        <v>2314309</v>
+        <v>2316880</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" s="2">
+        <v>46288.58326388889</v>
+      </c>
+      <c r="F11" s="1">
+        <v>9.0559097447817203E+21</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H11" s="14">
+        <v>155</v>
+      </c>
+      <c r="I11" s="9">
+        <f>Tabla1[[#This Row],[COSTO]]+50</f>
+        <v>205</v>
+      </c>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+    </row>
+    <row r="12" spans="1:11" ht="22.2" hidden="1" thickBot="1">
+      <c r="A12" s="1">
+        <v>2314309</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E12" s="2">
         <v>46287.342395833337</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F12" s="1">
         <v>2.0558981606127001E+21</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H12" s="1">
         <v>271</v>
       </c>
-      <c r="I11" s="4">
+      <c r="I12" s="4">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
         <v>321</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="39" thickBot="1">
-      <c r="A12" s="1">
+    <row r="13" spans="1:11" ht="39" thickBot="1">
+      <c r="A13" s="1">
         <v>2313907</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E13" s="2">
         <v>46286.680763888886</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F13" s="1">
         <v>3.0558981606127001E+21</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="14">
+      <c r="H13" s="14">
         <v>164</v>
       </c>
-      <c r="I12" s="9">
+      <c r="I13" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
         <v>214</v>
-      </c>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-    </row>
-    <row r="13" spans="1:11" ht="58.2" thickBot="1">
-      <c r="A13" s="1">
-        <v>2312903</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E13" s="2">
-        <v>46286.505462962959</v>
-      </c>
-      <c r="F13" s="1">
-        <v>5.5898160612700701E+19</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" s="14">
-        <v>310</v>
-      </c>
-      <c r="I13" s="9">
-        <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>360</v>
       </c>
       <c r="J13" s="11"/>
       <c r="K13" s="11"/>
     </row>
     <row r="14" spans="1:11" ht="58.2" thickBot="1">
       <c r="A14" s="1">
-        <v>2312796</v>
+        <v>2312903</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E14" s="2">
-        <v>46286.48704861111</v>
+        <v>46286.505462962959</v>
       </c>
       <c r="F14" s="1">
-        <v>3.0559097447817198E+21</v>
+        <v>5.5898160612700701E+19</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H14" s="14">
-        <v>155</v>
+        <v>310</v>
       </c>
       <c r="I14" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>205</v>
+        <v>360</v>
       </c>
       <c r="J14" s="11"/>
       <c r="K14" s="11"/>
     </row>
-    <row r="15" spans="1:11" ht="15" thickBot="1">
+    <row r="15" spans="1:11" ht="58.2" thickBot="1">
       <c r="A15" s="1">
-        <v>2309136</v>
+        <v>2312796</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E15" s="2">
-        <v>46282.538715277777</v>
+        <v>46286.48704861111</v>
       </c>
       <c r="F15" s="1">
-        <v>5.0558981606126995E+21</v>
+        <v>3.0559097447817198E+21</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H15" s="14">
-        <v>190</v>
+        <v>155</v>
       </c>
       <c r="I15" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="J15" s="11"/>
       <c r="K15" s="11"/>
     </row>
     <row r="16" spans="1:11" ht="15" thickBot="1">
       <c r="A16" s="1">
-        <v>2308942</v>
+        <v>2309136</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E16" s="2">
-        <v>46282.501782407409</v>
+        <v>46282.538715277777</v>
       </c>
       <c r="F16" s="1">
-        <v>6.0558981606126995E+21</v>
+        <v>5.0558981606126995E+21</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H16" s="14">
-        <v>229</v>
+        <v>190</v>
       </c>
       <c r="I16" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>279</v>
+        <v>240</v>
       </c>
       <c r="J16" s="11"/>
       <c r="K16" s="11"/>
     </row>
     <row r="17" spans="1:11" ht="15" thickBot="1">
       <c r="A17" s="1">
-        <v>2308752</v>
+        <v>2308942</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E17" s="2">
-        <v>46282.467881944445</v>
+        <v>46282.501782407409</v>
       </c>
       <c r="F17" s="1">
-        <v>9.0558981606126995E+21</v>
+        <v>6.0558981606126995E+21</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H17" s="14">
-        <v>179</v>
+        <v>229</v>
       </c>
       <c r="I17" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>229</v>
+        <v>279</v>
       </c>
       <c r="J17" s="11"/>
       <c r="K17" s="11"/>
     </row>
     <row r="18" spans="1:11" ht="15" thickBot="1">
       <c r="A18" s="1">
-        <v>2308664</v>
+        <v>2308752</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E18" s="2">
-        <v>46282.450474537036</v>
+        <v>46282.467881944445</v>
       </c>
       <c r="F18" s="1">
-        <v>1.0558981606127001E+21</v>
+        <v>9.0558981606126995E+21</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H18" s="14">
-        <v>229</v>
+        <v>179</v>
       </c>
       <c r="I18" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>279</v>
+        <v>229</v>
       </c>
       <c r="J18" s="11"/>
       <c r="K18" s="11"/>
     </row>
     <row r="19" spans="1:11" ht="15" thickBot="1">
       <c r="A19" s="1">
-        <v>2307450</v>
+        <v>2308664</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E19" s="2">
-        <v>46280.594768518517</v>
+        <v>46282.450474537036</v>
       </c>
       <c r="F19" s="1">
-        <v>8.0558981606126995E+21</v>
+        <v>1.0558981606127001E+21</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H19" s="14">
-        <v>271</v>
+        <v>229</v>
       </c>
       <c r="I19" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>321</v>
+        <v>279</v>
       </c>
       <c r="J19" s="11"/>
       <c r="K19" s="11"/>
     </row>
     <row r="20" spans="1:11" ht="15" thickBot="1">
       <c r="A20" s="1">
-        <v>2307446</v>
+        <v>2307450</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E20" s="2">
-        <v>46280.593831018516</v>
+        <v>46280.594768518517</v>
       </c>
       <c r="F20" s="1">
-        <v>5.5898160612700701E+19</v>
+        <v>8.0558981606126995E+21</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H20" s="14">
-        <v>302</v>
+        <v>271</v>
       </c>
       <c r="I20" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>352</v>
+        <v>321</v>
       </c>
       <c r="J20" s="11"/>
       <c r="K20" s="11"/>
     </row>
     <row r="21" spans="1:11" ht="15" thickBot="1">
       <c r="A21" s="1">
-        <v>2307438</v>
+        <v>2307446</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>0</v>
@@ -2530,10 +2531,10 @@
         <v>2</v>
       </c>
       <c r="E21" s="2">
-        <v>46280.591377314813</v>
+        <v>46280.593831018516</v>
       </c>
       <c r="F21" s="1">
-        <v>4.0558981606127001E+21</v>
+        <v>5.5898160612700701E+19</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>9</v>
@@ -2550,133 +2551,133 @@
     </row>
     <row r="22" spans="1:11" ht="15" thickBot="1">
       <c r="A22" s="1">
-        <v>2304456</v>
+        <v>2307438</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E22" s="2">
-        <v>46279.455949074072</v>
+        <v>46280.591377314813</v>
       </c>
       <c r="F22" s="1">
-        <v>3.0558981606127001E+21</v>
+        <v>4.0558981606127001E+21</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H22" s="14">
-        <v>179</v>
+        <v>302</v>
       </c>
       <c r="I22" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>229</v>
+        <v>352</v>
       </c>
       <c r="J22" s="11"/>
       <c r="K22" s="11"/>
     </row>
     <row r="23" spans="1:11" ht="15" thickBot="1">
       <c r="A23" s="1">
-        <v>2304430</v>
+        <v>2304456</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E23" s="2">
-        <v>46279.4528125</v>
+        <v>46279.455949074072</v>
       </c>
       <c r="F23" s="1">
-        <v>9.0558981606126995E+21</v>
+        <v>3.0558981606127001E+21</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H23" s="14">
-        <v>414</v>
+        <v>179</v>
       </c>
       <c r="I23" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>464</v>
+        <v>229</v>
       </c>
       <c r="J23" s="11"/>
       <c r="K23" s="11"/>
     </row>
-    <row r="24" spans="1:11" ht="22.2" hidden="1" thickBot="1">
+    <row r="24" spans="1:11" ht="15" thickBot="1">
       <c r="A24" s="1">
-        <v>2303299</v>
+        <v>2304430</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E24" s="2">
+        <v>46279.4528125</v>
+      </c>
+      <c r="F24" s="1">
+        <v>9.0558981606126995E+21</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H24" s="14">
+        <v>414</v>
+      </c>
+      <c r="I24" s="9">
+        <f>Tabla1[[#This Row],[COSTO]]+50</f>
+        <v>464</v>
+      </c>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+    </row>
+    <row r="25" spans="1:11" ht="22.2" hidden="1" thickBot="1">
+      <c r="A25" s="1">
+        <v>2303299</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E25" s="2">
         <v>46277.375405092593</v>
       </c>
-      <c r="F24" s="1">
+      <c r="F25" s="1">
         <v>8.0558981606126995E+21</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="G25" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H25" s="1">
         <v>271</v>
       </c>
-      <c r="I24" s="4">
+      <c r="I25" s="4">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
         <v>321</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" ht="15" thickBot="1">
-      <c r="A25" s="1">
-        <v>2302573</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E25" s="2">
-        <v>46276.538518518515</v>
-      </c>
-      <c r="F25" s="1">
-        <v>3.0558981606127001E+21</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H25" s="14">
-        <v>302</v>
-      </c>
-      <c r="I25" s="9">
-        <f>Tabla1[[#This Row],[COSTO]]+50</f>
-        <v>352</v>
-      </c>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
     </row>
     <row r="26" spans="1:11" ht="15" thickBot="1">
       <c r="A26" s="1">
-        <v>2302572</v>
+        <v>2302573</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>0</v>
@@ -2688,10 +2689,10 @@
         <v>2</v>
       </c>
       <c r="E26" s="2">
-        <v>46276.53769675926</v>
+        <v>46276.538518518515</v>
       </c>
       <c r="F26" s="1">
-        <v>5.0558981606126995E+21</v>
+        <v>3.0558981606127001E+21</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>9</v>
@@ -2699,33 +2700,65 @@
       <c r="H26" s="14">
         <v>302</v>
       </c>
-      <c r="I26" s="10">
+      <c r="I26" s="9">
         <f>Tabla1[[#This Row],[COSTO]]+50</f>
         <v>352</v>
       </c>
       <c r="J26" s="11"/>
       <c r="K26" s="11"/>
     </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="6"/>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="17">
-        <f>SUBTOTAL(9,I2:I26)</f>
-        <v>6730</v>
-      </c>
-      <c r="J27" s="12">
-        <f>SUBTOTAL(9,J2:J26)</f>
+    <row r="27" spans="1:11" ht="15" thickBot="1">
+      <c r="A27" s="1">
+        <v>2302572</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E27" s="2">
+        <v>46276.53769675926</v>
+      </c>
+      <c r="F27" s="1">
+        <v>5.0558981606126995E+21</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H27" s="14">
+        <v>302</v>
+      </c>
+      <c r="I27" s="10">
+        <f>Tabla1[[#This Row],[COSTO]]+50</f>
+        <v>352</v>
+      </c>
+      <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="17">
+        <f>SUBTOTAL(9,I2:I27)</f>
+        <v>6957</v>
+      </c>
+      <c r="J28" s="12">
+        <f>SUBTOTAL(9,J2:J27)</f>
         <v>5318</v>
       </c>
-      <c r="K27" s="12">
+      <c r="K28" s="12">
         <f>Tabla1[[#Totals],[SALDO]]-Tabla1[[#Totals],[PRECIO]]</f>
-        <v>-1412</v>
+        <v>-1639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>